<commit_message>
fix(narrative): (-1,-1) 认作「部件在图上没有位置」，不再刷 ITEM_PART_HOTSPOT_OUT_OF_RANGE
收录机的电池仓（RADIO_PART_03）和磁带（RADIO_PART_04）在这版美术里根本看不到
——磁带仓盖是卡死的，电池仓没画——所以配表里给了 (-1,-1)，靠详情页下方的按钮列表
进入（ItemPage 的 hotCount/listCount 分流本来就支持）。

校验器原来只认 0~1，一进战斗就 Error 刷屏。改成：两个都负数 = 白名单放行；
只有一半是负数的才算配错。配表表头注释同步写明这条约定。
</commit_message>
<xml_diff>
--- a/GameConfig/Datas/叙事物品部件配置表.xlsx
+++ b/GameConfig/Datas/叙事物品部件配置表.xlsx
@@ -563,12 +563,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>图片热点横坐标，归一化0到1</t>
+          <t>图片热点横坐标，归一化0到1；(-1,-1)表示这个部件在图上没有位置，改走详情页按钮列表</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>图片热点纵坐标，归一化0到1</t>
+          <t>图片热点纵坐标，归一化0到1（从下往上）；(-1,-1)同上</t>
         </is>
       </c>
     </row>

</xml_diff>